<commit_message>
Actualizar matriz y seeder: restringir eliminacion definitiva al Admin (exclusivo Super Admin)
</commit_message>
<xml_diff>
--- a/Matriz_Roles_y_Permisos_SGI.xlsx
+++ b/Matriz_Roles_y_Permisos_SGI.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="131">
   <si>
     <t>SGI - SISTEMA DE GESTIÓN DE INVENTARIOS | GRUPO NODO</t>
   </si>
@@ -23,7 +23,7 @@
     <t>MATRIZ DE PERMISOS CRUD (CREAR, LEER, ACTUALIZAR, ELIMINAR) Y AUDITORÍA DE LOGS</t>
   </si>
   <si>
-    <t>Control de accesos y responsabilidades: Usuario Estándar, Auxiliar, Almacenista, Admin y Super Admin</t>
+    <t>Regla de Seguridad: El Administrador (Admin) NO puede borrar definitivamente nada. La eliminación es exclusiva del Super Admin.</t>
   </si>
   <si>
     <t>DIRECTORIO DE USUARIOS ACTIVOS Y JERARQUÍA DE ROLES</t>
@@ -34,14 +34,16 @@
   <si>
     <t>usuariopruebacorreogi@gmail.com
 ramon8t2@gmail.com
-siguevictor767@gmail.com</t>
+siguevictor767@gmail.com
+★ ÚNICO rol con facultad de eliminación / baja definitiva.</t>
   </si>
   <si>
     <t>Admin (Nivel 2)</t>
   </si>
   <si>
     <t>Cuentas Directivas / Gerencia General
-(Control operativo total, sin permisos de eliminar Super Admin ni BD)</t>
+(Creación, Lectura y Actualización total.
+✖ NO puede borrar definitivamente nada).</t>
   </si>
   <si>
     <t>Almacenista (Nivel 3)</t>
@@ -49,7 +51,8 @@
   <si>
     <t>direccion.durga.dgi@gmail.com
 marce.nodo@gmail.com
-3523110518@uth.edu.mx</t>
+3523110518@uth.edu.mx
+(Operación de bodega: altas, existencias, vales. ✖ NO borra).</t>
   </si>
   <si>
     <t>Auxiliar (Nivel 4)</t>
@@ -57,14 +60,16 @@
   <si>
     <t>facturacion@naoproyectos.com
 gratservicios@gmail.com
-vconpuecomercializadora@gmail.com</t>
+vconpuecomercializadora@gmail.com
+(Apoyo operativo: consulta y consumo de insumos. ✖ NO borra).</t>
   </si>
   <si>
     <t>Usuario (Base / General)</t>
   </si>
   <si>
     <t>Cualquier empleado o cuenta básica
-(Solo consulta de perfil propio sin facultades de inventario)</t>
+(Solo consulta de su propio perfil.
+Sin privilegios operativos ni de inventario).</t>
   </si>
   <si>
     <t>MATRIZ OPERATIVA DE PERMISOS: CREAR, LEER, ACTUALIZAR Y ELIMINAR</t>
@@ -109,7 +114,7 @@
     <t>CREAR</t>
   </si>
   <si>
-    <t>Dar de alta nuevos activos fijos, asignar código interno, fotografía, valor comercial y custodio.</t>
+    <t>Dar de alta nuevos activos fijos, registrar serie, fotografía, costo comercial y asignar custodio.</t>
   </si>
   <si>
     <t>NO</t>
@@ -124,7 +129,7 @@
     <t>LEER</t>
   </si>
   <si>
-    <t>Consultar inventario activo, ver fichas técnicas, buscar por código de barras / QR y generar vales.</t>
+    <t>Consultar catálogo de activos, ver fichas técnicas, buscar por código de barras / QR y generar vales.</t>
   </si>
   <si>
     <t>Consulta de solo lectura (sin afectación de kardex)</t>
@@ -142,7 +147,7 @@
     <t>ELIMINAR</t>
   </si>
   <si>
-    <t>Dar de baja el bien por extravío, daño irreparable u obsolescencia (exige motivo y acta digital).</t>
+    <t>Dar de baja definitiva el activo por extravío, daño irreparable u obsolescencia (Exclusivo Super Admin con acta).</t>
   </si>
   <si>
     <t>Genera Log: Baja de Producto (con justificación obligatoria)</t>
@@ -169,7 +174,7 @@
     <t>Genera Log: Reabastecimiento de Existencias (suma a kardex)</t>
   </si>
   <si>
-    <t>Descartar consumible del catálogo o registrar ajuste por merma, derrame o caducidad.</t>
+    <t>Eliminar insumo del catálogo o purga por merma/caducidad grave (Exclusivo Super Admin).</t>
   </si>
   <si>
     <t>Genera Log: Baja / Merma de Insumo (con justificación)</t>
@@ -205,7 +210,7 @@
     <t>Genera Log: Actualización de Producto / Precios</t>
   </si>
   <si>
-    <t>Dar de baja producto comercial o registrar devolución por defecto a proveedor.</t>
+    <t>Dar de baja definitiva producto comercial o registrar devolución por defecto a proveedor (Exclusivo Super Admin).</t>
   </si>
   <si>
     <t>Genera Log: Baja / Devolución Comercial</t>
@@ -214,7 +219,7 @@
     <t>4. Vehículos y Flotilla</t>
   </si>
   <si>
-    <t>Dar de alta vehículo en flotilla con número de serie VIN, placas, marca, modelo y seguro.</t>
+    <t>Dar de alta vehículo en flotilla con número de serie VIN, placas, marca, modelo y póliza.</t>
   </si>
   <si>
     <t>Genera Log: Alta de Vehículo (categoría: vehiculos)</t>
@@ -229,7 +234,7 @@
     <t>Genera Log: Actualización / Reasignación Vehicular</t>
   </si>
   <si>
-    <t>Dar de baja unidad por siniestro total, venta de activo o término de arrendamiento.</t>
+    <t>Dar de baja definitiva vehículo por siniestro total, venta o término de arrendamiento (Exclusivo Super Admin con acta).</t>
   </si>
   <si>
     <t>Genera Log: Baja de Unidad Vehicular (con acta/finiquito)</t>
@@ -271,7 +276,7 @@
     <t>Genera Log: Modificación de Cuenta / Rol</t>
   </si>
   <si>
-    <t>Desactivar o suspender cuentas de usuario (Super Admin protegido contra desactivación).</t>
+    <t>Eliminar o suspender cuentas de usuario del sistema (Facultad exclusiva de Super Admin).</t>
   </si>
   <si>
     <t>Genera Log: Desactivación de Usuario</t>
@@ -295,7 +300,7 @@
     <t>Genera Log: Modificación de Permisos de Rol</t>
   </si>
   <si>
-    <t>Desactivar o eliminar roles existentes.</t>
+    <t>Desactivar o eliminar roles estructurales del sistema (Exclusivo Super Admin).</t>
   </si>
   <si>
     <t>Genera Log: Eliminación de Rol</t>
@@ -319,7 +324,7 @@
     <t>Genera Log: Actualización de Empresa</t>
   </si>
   <si>
-    <t>Desactivar empresas del catálogo activo.</t>
+    <t>Eliminar o desactivar empresas del catálogo oficial (Exclusivo Super Admin).</t>
   </si>
   <si>
     <t>Genera Log: Desactivación de Empresa</t>
@@ -343,7 +348,7 @@
     <t>Genera Log: Actualización de Ubicación</t>
   </si>
   <si>
-    <t>Desactivar o clausurar ubicaciones del catálogo.</t>
+    <t>Eliminar o clausurar bodegas y ubicaciones del sistema (Exclusivo Super Admin).</t>
   </si>
   <si>
     <t>Genera Log: Desactivación de Ubicación</t>
@@ -367,7 +372,7 @@
     <t>Genera Log: Modificación de Categoría</t>
   </si>
   <si>
-    <t>Desactivar categorías o etiquetas del catálogo.</t>
+    <t>Eliminar categorías o etiquetas del catálogo (Exclusivo Super Admin).</t>
   </si>
   <si>
     <t>Genera Log: Eliminación de Categoría</t>
@@ -409,13 +414,16 @@
     <t>Inmutable: Ningún rol puede borrar el historial de auditoría</t>
   </si>
   <si>
-    <t>RESUMEN TÉCNICO DE LOGS DE AUDITORÍA (TABLA `movimientos`)</t>
-  </si>
-  <si>
-    <t>DISPARADORES AUTOMÁTICOS: El sistema genera una fila inmutable de auditoría cada vez que un usuario: 1) Crea un activo o vehículo (Alta), 2) Modifica información o fotografías (Edición), 3) Da de baja un activo por descarte (Baja con justificación y acta), o 4) Consume consumibles (Consumo con cantidad y motivo).</t>
-  </si>
-  <si>
-    <t>ESTRUCTURA DE CAMPOS REGISTRADOS: `id` (Folio autoincremental) | `id_user` (Usuario autenticado responsable) | `id_producto` (Identificador del bien afectado) | `categoria` (fijos, consumibles, compraventa, vehiculos, sistema) | `accion` (Tipo de evento) | `comentario` (Motivo/justificante) | `documentacion` (Evidencia digital/foto) | `created_at` (Timestamp exacto).</t>
+    <t>RESUMEN TÉCNICO DE AUDITORÍA Y REGLAS DE ELIMINACIÓN</t>
+  </si>
+  <si>
+    <t>REGLA ESTRICTA DE BORRADO: El rol Administrador (Admin) NO tiene permitido eliminar ni dar de baja definitivamente ningún registro en el sistema (activos, consumibles, compra-venta, vehículos, empresas, ubicaciones, categorías, usuarios o roles). Dicha facultad queda restringida de manera exclusiva al Super Admin.</t>
+  </si>
+  <si>
+    <t>DISPARADORES AUTOMÁTICOS DE LOGS: Se genera una fila inmutable de auditoría cada vez que: 1) Se crea un activo o vehículo (Alta), 2) Se modifica información o fotos (Edición), 3) Se da de baja un activo (Baja justificada con acta), o 4) Se consumen existencias (Consumo con cantidad y motivo).</t>
+  </si>
+  <si>
+    <t>ESTRUCTURA DE CAMPOS REGISTRADOS EN BD: `id` (Folio único) | `id_user` (Usuario autenticado responsable) | `id_producto` (Identificador del bien) | `categoria` (fijos, consumibles, compraventa, vehiculos, sistema) | `accion` (Tipo de evento) | `comentario` (Motivo/justificante) | `documentacion` (Evidencia digital/foto) | `created_at` (Timestamp exacto).</t>
   </si>
 </sst>
 </file>
@@ -423,7 +431,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
   <numFmts count="0"/>
-  <fonts count="26">
+  <fonts count="27">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -452,12 +460,12 @@
       <name val="Calibri"/>
     </font>
     <font>
-      <b val="0"/>
+      <b val="1"/>
       <i val="1"/>
       <strike val="0"/>
       <u val="none"/>
       <sz val="10"/>
-      <color rgb="FF64748B"/>
+      <color rgb="FFDC2626"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -646,6 +654,15 @@
       <strike val="0"/>
       <u val="none"/>
       <sz val="9"/>
+      <color rgb="FF991B1B"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="8.5"/>
       <color rgb="FF0F172A"/>
       <name val="Calibri"/>
     </font>
@@ -751,7 +768,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -791,6 +808,21 @@
     </border>
     <border>
       <left style="thin">
+        <color rgb="FFEF4444"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFEF4444"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFEF4444"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFEF4444"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
         <color rgb="FF38BDF8"/>
       </left>
       <right style="thin">
@@ -808,7 +840,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
       <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
@@ -914,10 +946,13 @@
     <xf xfId="0" fontId="23" numFmtId="0" fillId="3" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="24" numFmtId="0" fillId="15" borderId="3" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="24" numFmtId="0" fillId="10" borderId="3" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="25" numFmtId="0" fillId="12" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="25" numFmtId="0" fillId="15" borderId="4" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="26" numFmtId="0" fillId="12" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
   </cellXfs>
@@ -1219,7 +1254,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:J58"/>
+  <dimension ref="A1:J59"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -1462,11 +1497,11 @@
       <c r="F15" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="G15" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="H15" s="18" t="s">
-        <v>29</v>
+      <c r="G15" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="H15" s="17" t="s">
+        <v>28</v>
       </c>
       <c r="I15" s="18" t="s">
         <v>29</v>
@@ -1593,8 +1628,8 @@
       <c r="G19" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="H19" s="18" t="s">
-        <v>29</v>
+      <c r="H19" s="17" t="s">
+        <v>28</v>
       </c>
       <c r="I19" s="18" t="s">
         <v>29</v>
@@ -1753,8 +1788,8 @@
       <c r="G24" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="H24" s="18" t="s">
-        <v>29</v>
+      <c r="H24" s="17" t="s">
+        <v>28</v>
       </c>
       <c r="I24" s="18" t="s">
         <v>29</v>
@@ -1881,8 +1916,8 @@
       <c r="G28" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="H28" s="18" t="s">
-        <v>29</v>
+      <c r="H28" s="17" t="s">
+        <v>28</v>
       </c>
       <c r="I28" s="18" t="s">
         <v>29</v>
@@ -2041,8 +2076,8 @@
       <c r="G33" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="H33" s="18" t="s">
-        <v>78</v>
+      <c r="H33" s="17" t="s">
+        <v>28</v>
       </c>
       <c r="I33" s="18" t="s">
         <v>29</v>
@@ -2297,8 +2332,8 @@
       <c r="G41" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="H41" s="18" t="s">
-        <v>29</v>
+      <c r="H41" s="17" t="s">
+        <v>28</v>
       </c>
       <c r="I41" s="18" t="s">
         <v>29</v>
@@ -2425,8 +2460,8 @@
       <c r="G45" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="H45" s="18" t="s">
-        <v>29</v>
+      <c r="H45" s="17" t="s">
+        <v>28</v>
       </c>
       <c r="I45" s="18" t="s">
         <v>29</v>
@@ -2553,8 +2588,8 @@
       <c r="G49" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="H49" s="18" t="s">
-        <v>29</v>
+      <c r="H49" s="17" t="s">
+        <v>28</v>
       </c>
       <c r="I49" s="18" t="s">
         <v>29</v>
@@ -2696,7 +2731,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="57" spans="1:10" customHeight="1" ht="32">
+    <row r="57" spans="1:10" customHeight="1" ht="30">
       <c r="A57" s="37" t="s">
         <v>128</v>
       </c>
@@ -2723,6 +2758,20 @@
       <c r="H58" s="38"/>
       <c r="I58" s="38"/>
       <c r="J58" s="38"/>
+    </row>
+    <row r="59" spans="1:10" customHeight="1" ht="28">
+      <c r="A59" s="39" t="s">
+        <v>130</v>
+      </c>
+      <c r="B59" s="39"/>
+      <c r="C59" s="39"/>
+      <c r="D59" s="39"/>
+      <c r="E59" s="39"/>
+      <c r="F59" s="39"/>
+      <c r="G59" s="39"/>
+      <c r="H59" s="39"/>
+      <c r="I59" s="39"/>
+      <c r="J59" s="39"/>
     </row>
   </sheetData>
   <mergeCells>
@@ -2738,6 +2787,7 @@
     <mergeCell ref="I7:J8"/>
     <mergeCell ref="A57:J57"/>
     <mergeCell ref="A58:J58"/>
+    <mergeCell ref="A59:J59"/>
   </mergeCells>
   <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Soporte para proxies/ngrok y redireccion GET a inicio de sesion
</commit_message>
<xml_diff>
--- a/Matriz_Roles_y_Permisos_SGI.xlsx
+++ b/Matriz_Roles_y_Permisos_SGI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\SGI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AC38619-7F0E-41BA-AADA-75139D4FDC7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD87DA19-A0D1-4EE0-9652-8878E5023F3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -86,9 +86,6 @@
     <t>5. Gestión de Usuarios</t>
   </si>
   <si>
-    <t>SÍ (Protegido)</t>
-  </si>
-  <si>
     <t>SÍ (Total)</t>
   </si>
   <si>
@@ -102,6 +99,9 @@
   </si>
   <si>
     <t>9. Categorías y Etiquetas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SÍ </t>
   </si>
 </sst>
 </file>
@@ -1163,11 +1163,11 @@
       <c r="E23" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="F23" s="7" t="s">
+      <c r="F23" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="G23" s="7" t="s">
         <v>21</v>
-      </c>
-      <c r="G23" s="7" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1198,7 +1198,7 @@
         <v>23</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>9</v>
@@ -1221,7 +1221,7 @@
         <v>24</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C26" s="10" t="s">
         <v>12</v>
@@ -1244,7 +1244,7 @@
         <v>25</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C27" s="11" t="s">
         <v>13</v>
@@ -1267,7 +1267,7 @@
         <v>26</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C28" s="12" t="s">
         <v>14</v>
@@ -1290,7 +1290,7 @@
         <v>27</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C29" s="5" t="s">
         <v>9</v>
@@ -1313,7 +1313,7 @@
         <v>28</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C30" s="10" t="s">
         <v>12</v>
@@ -1336,7 +1336,7 @@
         <v>29</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C31" s="11" t="s">
         <v>13</v>
@@ -1359,7 +1359,7 @@
         <v>30</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C32" s="12" t="s">
         <v>14</v>
@@ -1382,7 +1382,7 @@
         <v>31</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C33" s="5" t="s">
         <v>9</v>
@@ -1405,7 +1405,7 @@
         <v>32</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C34" s="10" t="s">
         <v>12</v>
@@ -1428,7 +1428,7 @@
         <v>33</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C35" s="11" t="s">
         <v>13</v>
@@ -1451,7 +1451,7 @@
         <v>34</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C36" s="12" t="s">
         <v>14</v>
@@ -1474,7 +1474,7 @@
         <v>35</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C37" s="5" t="s">
         <v>9</v>
@@ -1497,7 +1497,7 @@
         <v>36</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C38" s="10" t="s">
         <v>12</v>
@@ -1520,7 +1520,7 @@
         <v>37</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C39" s="11" t="s">
         <v>13</v>
@@ -1543,7 +1543,7 @@
         <v>38</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C40" s="12" t="s">
         <v>14</v>

</xml_diff>